<commit_message>
Compare foundation-priced delivery options for ROM review
</commit_message>
<xml_diff>
--- a/docs/releases/proofs/2026-10-10-moves-demo-case-numbers-rom-workbook.xlsx
+++ b/docs/releases/proofs/2026-10-10-moves-demo-case-numbers-rom-workbook.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="186">
   <si>
     <t>ROM estimate — live formulas</t>
   </si>
@@ -314,7 +314,7 @@
     <t>rate = band ROL-024-LVL-06 indicative_bill_rate $406.25 × location LOC-DALLAS 1.00 × provider 1.00 = $406.25/hr</t>
   </si>
   <si>
-    <t>band rate_basis onshore_si_t1_benchmark (benchmark SI-T1, onshore); band confidence medium, approval global_starter_unapproved; location scarcity_multiplier not applied in this increment</t>
+    <t>band rate_basis onshore_si_t1_benchmark (benchmark SI-T1, onshore); band confidence medium, approval global_starter_unapproved; location scarcity_multiplier not applied in this increment; planning rates, not approved</t>
   </si>
   <si>
     <t>rate_band:ROL-023-LVL-07:indicative_bill_rate [Workforce_Taxonomy_Master.xlsx:Role Rate Card row RC-0066 (Internal Cost Model + Assumptions formula engine, recomputed — see script header)]</t>
@@ -456,6 +456,15 @@
   </si>
   <si>
     <t>ROM policy: no credit unless explicitly requested</t>
+  </si>
+  <si>
+    <t>Rate approval status</t>
+  </si>
+  <si>
+    <t>planning rates, not approved</t>
+  </si>
+  <si>
+    <t>Review every role band and delivery mapping before estimate approval</t>
   </si>
   <si>
     <t>Release R1 design status</t>
@@ -611,11 +620,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1958,7 +1973,7 @@
         <v>62</v>
       </c>
       <c r="B41">
-        <f>'Assumptions'!$B$11</f>
+        <f>'Assumptions'!$B$12</f>
         <v>0.75</v>
       </c>
     </row>
@@ -1967,7 +1982,7 @@
         <v>63</v>
       </c>
       <c r="B42">
-        <f>'Assumptions'!$B$12</f>
+        <f>'Assumptions'!$B$13</f>
         <v>1.5</v>
       </c>
     </row>
@@ -2243,7 +2258,7 @@
         <v>62</v>
       </c>
       <c r="B58">
-        <f>'Assumptions'!$B$14</f>
+        <f>'Assumptions'!$B$15</f>
         <v>0.75</v>
       </c>
     </row>
@@ -2252,7 +2267,7 @@
         <v>63</v>
       </c>
       <c r="B59">
-        <f>'Assumptions'!$B$15</f>
+        <f>'Assumptions'!$B$16</f>
         <v>1.5</v>
       </c>
     </row>
@@ -2528,7 +2543,7 @@
         <v>62</v>
       </c>
       <c r="B75">
-        <f>'Assumptions'!$B$17</f>
+        <f>'Assumptions'!$B$18</f>
         <v>0.75</v>
       </c>
     </row>
@@ -2537,7 +2552,7 @@
         <v>63</v>
       </c>
       <c r="B76">
-        <f>'Assumptions'!$B$18</f>
+        <f>'Assumptions'!$B$19</f>
         <v>1.5</v>
       </c>
     </row>
@@ -2703,10 +2718,25 @@
   <dimension ref="A1:R6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="18" width="18" customWidth="1"/>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="23" customWidth="1"/>
+    <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="52" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="44" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="44" customWidth="1"/>
+    <col min="13" max="15" width="18" customWidth="1"/>
+    <col min="16" max="16" width="27" customWidth="1"/>
+    <col min="17" max="17" width="62" customWidth="1"/>
+    <col min="18" max="18" width="58" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="32" customHeight="1" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>78</v>
       </c>
@@ -2728,19 +2758,19 @@
       <c r="G1" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="4" t="s">
         <v>82</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="4" t="s">
         <v>84</v>
       </c>
       <c r="K1" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="4" t="s">
         <v>86</v>
       </c>
       <c r="M1" s="3" t="s">
@@ -2752,17 +2782,17 @@
       <c r="O1" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="R1" s="4" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" ht="96" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2784,19 +2814,19 @@
       <c r="G2">
         <v>40625</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="5" t="s">
         <v>94</v>
       </c>
       <c r="I2">
         <v>1</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="5" t="s">
         <v>95</v>
       </c>
       <c r="K2">
         <v>1</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="5" t="s">
         <v>96</v>
       </c>
       <c r="M2">
@@ -2810,17 +2840,17 @@
       <c r="O2" t="s">
         <v>97</v>
       </c>
-      <c r="P2" t="s">
+      <c r="P2" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="Q2" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="R2" t="s">
+      <c r="R2" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" ht="96" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2842,19 +2872,19 @@
       <c r="G3">
         <v>34938</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="5" t="s">
         <v>100</v>
       </c>
       <c r="I3">
         <v>1</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="5" t="s">
         <v>95</v>
       </c>
       <c r="K3">
         <v>1</v>
       </c>
-      <c r="L3" t="s">
+      <c r="L3" s="5" t="s">
         <v>96</v>
       </c>
       <c r="M3">
@@ -2868,17 +2898,17 @@
       <c r="O3" t="s">
         <v>97</v>
       </c>
-      <c r="P3" t="s">
+      <c r="P3" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="Q3" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="R3" t="s">
+      <c r="R3" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" ht="96" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2900,19 +2930,19 @@
       <c r="G4">
         <v>29250</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="5" t="s">
         <v>102</v>
       </c>
       <c r="I4">
         <v>1</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="5" t="s">
         <v>95</v>
       </c>
       <c r="K4">
         <v>1</v>
       </c>
-      <c r="L4" t="s">
+      <c r="L4" s="5" t="s">
         <v>96</v>
       </c>
       <c r="M4">
@@ -2926,17 +2956,17 @@
       <c r="O4" t="s">
         <v>97</v>
       </c>
-      <c r="P4" t="s">
+      <c r="P4" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="Q4" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="R4" t="s">
+      <c r="R4" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" ht="96" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2958,19 +2988,19 @@
       <c r="G5">
         <v>24750</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="5" t="s">
         <v>104</v>
       </c>
       <c r="I5">
         <v>1</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J5" s="5" t="s">
         <v>95</v>
       </c>
       <c r="K5">
         <v>1</v>
       </c>
-      <c r="L5" t="s">
+      <c r="L5" s="5" t="s">
         <v>96</v>
       </c>
       <c r="M5">
@@ -2984,17 +3014,17 @@
       <c r="O5" t="s">
         <v>97</v>
       </c>
-      <c r="P5" t="s">
+      <c r="P5" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="Q5" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="R5" t="s">
+      <c r="R5" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" ht="96" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>40</v>
       </c>
@@ -3014,6 +3044,12 @@
         <f>ROUND(SUM(F2:F5),4)</f>
         <v>10</v>
       </c>
+      <c r="H6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="L6" s="5"/>
+      <c r="P6" s="5"/>
+      <c r="Q6" s="5"/>
+      <c r="R6" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3296,10 +3332,14 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="5" width="18" customWidth="1"/>
+    <col min="1" max="1" width="46" customWidth="1"/>
+    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="68" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3460,13 +3500,13 @@
         <v>147</v>
       </c>
       <c r="B10" t="s">
-        <v>37</v>
+        <v>148</v>
       </c>
       <c r="C10" t="s">
         <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="E10" t="s">
         <v>34</v>
@@ -3474,16 +3514,16 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>148</v>
-      </c>
-      <c r="B11">
-        <v>0.75</v>
+        <v>150</v>
+      </c>
+      <c r="B11" t="s">
+        <v>37</v>
       </c>
       <c r="C11" t="s">
-        <v>130</v>
+        <v>34</v>
       </c>
       <c r="D11" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="E11" t="s">
         <v>34</v>
@@ -3491,16 +3531,16 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B12">
-        <v>1.5</v>
+        <v>0.75</v>
       </c>
       <c r="C12" t="s">
         <v>130</v>
       </c>
       <c r="D12" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E12" t="s">
         <v>34</v>
@@ -3508,16 +3548,16 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>151</v>
-      </c>
-      <c r="B13" t="s">
-        <v>37</v>
+        <v>153</v>
+      </c>
+      <c r="B13">
+        <v>1.5</v>
       </c>
       <c r="C13" t="s">
-        <v>34</v>
+        <v>130</v>
       </c>
       <c r="D13" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="E13" t="s">
         <v>34</v>
@@ -3525,16 +3565,16 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>152</v>
-      </c>
-      <c r="B14">
-        <v>0.75</v>
+        <v>154</v>
+      </c>
+      <c r="B14" t="s">
+        <v>37</v>
       </c>
       <c r="C14" t="s">
-        <v>130</v>
+        <v>34</v>
       </c>
       <c r="D14" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="E14" t="s">
         <v>34</v>
@@ -3542,16 +3582,16 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B15">
-        <v>1.5</v>
+        <v>0.75</v>
       </c>
       <c r="C15" t="s">
         <v>130</v>
       </c>
       <c r="D15" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E15" t="s">
         <v>34</v>
@@ -3559,16 +3599,16 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>154</v>
-      </c>
-      <c r="B16" t="s">
-        <v>37</v>
+        <v>156</v>
+      </c>
+      <c r="B16">
+        <v>1.5</v>
       </c>
       <c r="C16" t="s">
-        <v>34</v>
+        <v>130</v>
       </c>
       <c r="D16" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="E16" t="s">
         <v>34</v>
@@ -3576,16 +3616,16 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>155</v>
-      </c>
-      <c r="B17">
-        <v>0.75</v>
+        <v>157</v>
+      </c>
+      <c r="B17" t="s">
+        <v>37</v>
       </c>
       <c r="C17" t="s">
-        <v>130</v>
+        <v>34</v>
       </c>
       <c r="D17" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="E17" t="s">
         <v>34</v>
@@ -3593,16 +3633,16 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B18">
-        <v>1.5</v>
+        <v>0.75</v>
       </c>
       <c r="C18" t="s">
         <v>130</v>
       </c>
       <c r="D18" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E18" t="s">
         <v>34</v>
@@ -3610,433 +3650,450 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B19">
+        <v>1.5</v>
+      </c>
+      <c r="C19" t="s">
+        <v>130</v>
+      </c>
+      <c r="D19" t="s">
+        <v>152</v>
+      </c>
+      <c r="E19" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>160</v>
+      </c>
+      <c r="B20">
         <f>'Component Library'!$C$2</f>
         <v>36</v>
       </c>
-      <c r="C19" t="s">
-        <v>158</v>
-      </c>
-      <c r="D19" t="s">
+      <c r="C20" t="s">
+        <v>161</v>
+      </c>
+      <c r="D20" t="s">
         <v>16</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E20" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>159</v>
-      </c>
-      <c r="B20">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>162</v>
+      </c>
+      <c r="B21">
         <f>'Component Library'!$C$3</f>
         <v>8</v>
       </c>
-      <c r="C20" t="s">
-        <v>158</v>
-      </c>
-      <c r="D20" t="s">
+      <c r="C21" t="s">
+        <v>161</v>
+      </c>
+      <c r="D21" t="s">
         <v>19</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E21" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>160</v>
-      </c>
-      <c r="B21">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>163</v>
+      </c>
+      <c r="B22">
         <f>'Component Library'!$C$4</f>
         <v>28</v>
       </c>
-      <c r="C21" t="s">
-        <v>158</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="C22" t="s">
+        <v>161</v>
+      </c>
+      <c r="D22" t="s">
         <v>21</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E22" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>161</v>
-      </c>
-      <c r="B22">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>164</v>
+      </c>
+      <c r="B23">
         <f>'Component Library'!$C$5</f>
         <v>24</v>
       </c>
-      <c r="C22" t="s">
-        <v>158</v>
-      </c>
-      <c r="D22" t="s">
+      <c r="C23" t="s">
+        <v>161</v>
+      </c>
+      <c r="D23" t="s">
         <v>23</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E23" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>162</v>
-      </c>
-      <c r="B23">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>165</v>
+      </c>
+      <c r="B24">
         <f>'Component Library'!$C$6</f>
         <v>3</v>
       </c>
-      <c r="C23" t="s">
-        <v>158</v>
-      </c>
-      <c r="D23" t="s">
+      <c r="C24" t="s">
+        <v>161</v>
+      </c>
+      <c r="D24" t="s">
         <v>25</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E24" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>163</v>
-      </c>
-      <c r="B24">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>166</v>
+      </c>
+      <c r="B25">
         <f>'Component Library'!$C$7</f>
         <v>2</v>
       </c>
-      <c r="C24" t="s">
-        <v>158</v>
-      </c>
-      <c r="D24" t="s">
+      <c r="C25" t="s">
+        <v>161</v>
+      </c>
+      <c r="D25" t="s">
         <v>27</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E25" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>164</v>
-      </c>
-      <c r="B25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>167</v>
+      </c>
+      <c r="B26">
         <f>'Estimate'!$E$5</f>
         <v>20</v>
       </c>
-      <c r="C25" t="s">
-        <v>165</v>
-      </c>
-      <c r="D25" t="s">
+      <c r="C26" t="s">
+        <v>168</v>
+      </c>
+      <c r="D26" t="s">
         <v>137</v>
       </c>
-      <c r="E25" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>166</v>
-      </c>
-      <c r="B26">
+      <c r="E26" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>169</v>
+      </c>
+      <c r="B27">
         <f>'Estimate'!$E$6</f>
         <v>80</v>
       </c>
-      <c r="C26" t="s">
-        <v>165</v>
-      </c>
-      <c r="D26" t="s">
+      <c r="C27" t="s">
+        <v>168</v>
+      </c>
+      <c r="D27" t="s">
         <v>137</v>
       </c>
-      <c r="E26" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>167</v>
-      </c>
-      <c r="B27">
+      <c r="E27" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>170</v>
+      </c>
+      <c r="B28">
         <f>'Estimate'!$E$7</f>
         <v>55</v>
       </c>
-      <c r="C27" t="s">
-        <v>165</v>
-      </c>
-      <c r="D27" t="s">
+      <c r="C28" t="s">
+        <v>168</v>
+      </c>
+      <c r="D28" t="s">
         <v>137</v>
       </c>
-      <c r="E27" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>168</v>
-      </c>
-      <c r="B28">
+      <c r="E28" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>171</v>
+      </c>
+      <c r="B29">
         <f>'Estimate'!$E$8</f>
         <v>25</v>
       </c>
-      <c r="C28" t="s">
-        <v>165</v>
-      </c>
-      <c r="D28" t="s">
+      <c r="C29" t="s">
+        <v>168</v>
+      </c>
+      <c r="D29" t="s">
         <v>137</v>
       </c>
-      <c r="E28" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>169</v>
-      </c>
-      <c r="B29">
+      <c r="E29" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>172</v>
+      </c>
+      <c r="B30">
         <f>'Estimate'!$E$9</f>
         <v>200</v>
       </c>
-      <c r="C29" t="s">
-        <v>165</v>
-      </c>
-      <c r="D29" t="s">
+      <c r="C30" t="s">
+        <v>168</v>
+      </c>
+      <c r="D30" t="s">
         <v>137</v>
       </c>
-      <c r="E29" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>170</v>
-      </c>
-      <c r="B30">
+      <c r="E30" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>173</v>
+      </c>
+      <c r="B31">
         <f>'Estimate'!$E$10</f>
         <v>255</v>
       </c>
-      <c r="C30" t="s">
-        <v>165</v>
-      </c>
-      <c r="D30" t="s">
+      <c r="C31" t="s">
+        <v>168</v>
+      </c>
+      <c r="D31" t="s">
         <v>137</v>
       </c>
-      <c r="E30" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>171</v>
-      </c>
-      <c r="B31">
+      <c r="E31" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>174</v>
+      </c>
+      <c r="B32">
         <f>'Estimate'!$E$11</f>
         <v>18</v>
       </c>
-      <c r="C31" t="s">
-        <v>165</v>
-      </c>
-      <c r="D31" t="s">
+      <c r="C32" t="s">
+        <v>168</v>
+      </c>
+      <c r="D32" t="s">
         <v>137</v>
       </c>
-      <c r="E31" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>172</v>
-      </c>
-      <c r="B32">
+      <c r="E32" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>175</v>
+      </c>
+      <c r="B33">
         <f>'Estimate'!$E$12</f>
         <v>80</v>
       </c>
-      <c r="C32" t="s">
-        <v>165</v>
-      </c>
-      <c r="D32" t="s">
+      <c r="C33" t="s">
+        <v>168</v>
+      </c>
+      <c r="D33" t="s">
         <v>137</v>
       </c>
-      <c r="E32" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>173</v>
-      </c>
-      <c r="B33">
+      <c r="E33" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>176</v>
+      </c>
+      <c r="B34">
         <f>'Estimate'!$E$13</f>
         <v>45</v>
       </c>
-      <c r="C33" t="s">
-        <v>165</v>
-      </c>
-      <c r="D33" t="s">
+      <c r="C34" t="s">
+        <v>168</v>
+      </c>
+      <c r="D34" t="s">
         <v>137</v>
       </c>
-      <c r="E33" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>174</v>
-      </c>
-      <c r="B34">
+      <c r="E34" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>177</v>
+      </c>
+      <c r="B35">
         <f>'Estimate'!$E$14</f>
         <v>30</v>
       </c>
-      <c r="C34" t="s">
-        <v>165</v>
-      </c>
-      <c r="D34" t="s">
+      <c r="C35" t="s">
+        <v>168</v>
+      </c>
+      <c r="D35" t="s">
         <v>137</v>
       </c>
-      <c r="E34" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>175</v>
-      </c>
-      <c r="B35">
+      <c r="E35" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>178</v>
+      </c>
+      <c r="B36">
         <f>'Estimate'!$E$15</f>
         <v>150</v>
       </c>
-      <c r="C35" t="s">
-        <v>165</v>
-      </c>
-      <c r="D35" t="s">
+      <c r="C36" t="s">
+        <v>168</v>
+      </c>
+      <c r="D36" t="s">
         <v>137</v>
       </c>
-      <c r="E35" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>176</v>
-      </c>
-      <c r="B36">
+      <c r="E36" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>179</v>
+      </c>
+      <c r="B37">
         <f>'Estimate'!$E$16</f>
         <v>220</v>
       </c>
-      <c r="C36" t="s">
-        <v>165</v>
-      </c>
-      <c r="D36" t="s">
+      <c r="C37" t="s">
+        <v>168</v>
+      </c>
+      <c r="D37" t="s">
         <v>137</v>
       </c>
-      <c r="E36" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>177</v>
-      </c>
-      <c r="B37">
+      <c r="E37" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>180</v>
+      </c>
+      <c r="B38">
         <f>'Estimate'!$E$17</f>
         <v>8</v>
       </c>
-      <c r="C37" t="s">
-        <v>165</v>
-      </c>
-      <c r="D37" t="s">
+      <c r="C38" t="s">
+        <v>168</v>
+      </c>
+      <c r="D38" t="s">
         <v>137</v>
       </c>
-      <c r="E37" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>178</v>
-      </c>
-      <c r="B38">
+      <c r="E38" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>181</v>
+      </c>
+      <c r="B39">
         <f>'Estimate'!$E$18</f>
         <v>65</v>
       </c>
-      <c r="C38" t="s">
-        <v>165</v>
-      </c>
-      <c r="D38" t="s">
+      <c r="C39" t="s">
+        <v>168</v>
+      </c>
+      <c r="D39" t="s">
         <v>137</v>
       </c>
-      <c r="E38" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>179</v>
-      </c>
-      <c r="B39">
+      <c r="E39" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>182</v>
+      </c>
+      <c r="B40">
         <f>'Estimate'!$E$19</f>
         <v>20</v>
       </c>
-      <c r="C39" t="s">
-        <v>165</v>
-      </c>
-      <c r="D39" t="s">
+      <c r="C40" t="s">
+        <v>168</v>
+      </c>
+      <c r="D40" t="s">
         <v>137</v>
       </c>
-      <c r="E39" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>180</v>
-      </c>
-      <c r="B40">
+      <c r="E40" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>183</v>
+      </c>
+      <c r="B41">
         <f>'Estimate'!$E$20</f>
         <v>8</v>
       </c>
-      <c r="C40" t="s">
-        <v>165</v>
-      </c>
-      <c r="D40" t="s">
+      <c r="C41" t="s">
+        <v>168</v>
+      </c>
+      <c r="D41" t="s">
         <v>137</v>
       </c>
-      <c r="E40" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>181</v>
-      </c>
-      <c r="B41">
+      <c r="E41" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>184</v>
+      </c>
+      <c r="B42">
         <f>'Estimate'!$E$21</f>
         <v>100</v>
       </c>
-      <c r="C41" t="s">
-        <v>165</v>
-      </c>
-      <c r="D41" t="s">
+      <c r="C42" t="s">
+        <v>168</v>
+      </c>
+      <c r="D42" t="s">
         <v>137</v>
       </c>
-      <c r="E41" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>182</v>
-      </c>
-      <c r="B42">
+      <c r="E42" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>185</v>
+      </c>
+      <c r="B43">
         <f>'Estimate'!$E$22</f>
         <v>130</v>
       </c>
-      <c r="C42" t="s">
-        <v>165</v>
-      </c>
-      <c r="D42" t="s">
+      <c r="C43" t="s">
+        <v>168</v>
+      </c>
+      <c r="D43" t="s">
         <v>137</v>
       </c>
-      <c r="E42" t="s">
+      <c r="E43" t="s">
         <v>34</v>
       </c>
     </row>

</xml_diff>